<commit_message>
version 47 - Adapt SW with 3NF DBMS and design document for tracing
</commit_message>
<xml_diff>
--- a/Documentation/API_Design/RESTFul_API.xlsx
+++ b/Documentation/API_Design/RESTFul_API.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8280"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Server APIs" sheetId="3" r:id="rId1"/>
@@ -176,7 +176,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="235">
   <si>
     <t>RESTfull API</t>
   </si>
@@ -1493,6 +1493,12 @@
   </si>
   <si>
     <t>ADMIN_OrderStatus_URL</t>
+  </si>
+  <si>
+    <t>API 25: Get Data from MongoDB and merge with MySQL Products</t>
+  </si>
+  <si>
+    <t>/api/admin/update_products_mysql</t>
   </si>
 </sst>
 </file>
@@ -1739,7 +1745,7 @@
       <charset val="0"/>
     </font>
   </fonts>
-  <fills count="42">
+  <fills count="43">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1785,6 +1791,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.25"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2252,7 +2264,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2276,16 +2288,16 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -2294,89 +2306,89 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2523,43 +2535,52 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2587,10 +2608,13 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2967,7 +2991,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.4"/>
   <cols>
     <col min="1" max="1" width="38.5833333333333" style="2" customWidth="1"/>
@@ -3012,7 +3036,7 @@
       </c>
       <c r="I2" s="12"/>
       <c r="J2" s="12"/>
-      <c r="K2" s="61" t="s">
+      <c r="K2" s="64" t="s">
         <v>7</v>
       </c>
     </row>
@@ -3039,7 +3063,7 @@
       <c r="J3" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="62"/>
+      <c r="K3" s="65"/>
     </row>
     <row r="4" s="2" customFormat="1" ht="54" customHeight="1" spans="1:11">
       <c r="A4" s="18" t="s">
@@ -3054,13 +3078,13 @@
       <c r="D4" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="75" t="s">
+      <c r="E4" s="79" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="75" t="s">
+      <c r="G4" s="79" t="s">
         <v>18</v>
       </c>
       <c r="H4" s="23" t="s">
@@ -3068,7 +3092,7 @@
       </c>
       <c r="I4" s="26"/>
       <c r="J4" s="26"/>
-      <c r="K4" s="76" t="s">
+      <c r="K4" s="80" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3085,13 +3109,13 @@
       <c r="D5" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="75" t="s">
+      <c r="E5" s="79" t="s">
         <v>24</v>
       </c>
       <c r="F5" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="75" t="s">
+      <c r="G5" s="79" t="s">
         <v>25</v>
       </c>
       <c r="H5" s="23" t="s">
@@ -3099,7 +3123,7 @@
       </c>
       <c r="I5" s="26"/>
       <c r="J5" s="26"/>
-      <c r="K5" s="64" t="s">
+      <c r="K5" s="67" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3115,16 +3139,16 @@
       </c>
       <c r="F6" s="26"/>
       <c r="G6" s="26"/>
-      <c r="H6" s="75" t="s">
+      <c r="H6" s="79" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="75" t="s">
+      <c r="I6" s="79" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="75" t="s">
+      <c r="J6" s="79" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="64" t="s">
+      <c r="K6" s="67" t="s">
         <v>31</v>
       </c>
     </row>
@@ -3135,7 +3159,7 @@
       <c r="D7" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="77" t="s">
+      <c r="E7" s="81" t="s">
         <v>33</v>
       </c>
       <c r="F7" s="27"/>
@@ -3145,7 +3169,7 @@
       </c>
       <c r="I7" s="26"/>
       <c r="J7" s="26"/>
-      <c r="K7" s="64" t="s">
+      <c r="K7" s="67" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3161,7 +3185,7 @@
       </c>
       <c r="F8" s="26"/>
       <c r="G8" s="26"/>
-      <c r="H8" s="78" t="s">
+      <c r="H8" s="82" t="s">
         <v>36</v>
       </c>
       <c r="I8" s="28" t="s">
@@ -3170,7 +3194,7 @@
       <c r="J8" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="K8" s="65" t="s">
+      <c r="K8" s="68" t="s">
         <v>39</v>
       </c>
     </row>
@@ -3184,7 +3208,7 @@
       <c r="E9" s="23"/>
       <c r="F9" s="26"/>
       <c r="G9" s="26"/>
-      <c r="H9" s="78" t="s">
+      <c r="H9" s="82" t="s">
         <v>41</v>
       </c>
       <c r="I9" s="28" t="s">
@@ -3193,7 +3217,7 @@
       <c r="J9" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="K9" s="65" t="s">
+      <c r="K9" s="68" t="s">
         <v>43</v>
       </c>
     </row>
@@ -3220,7 +3244,7 @@
       </c>
       <c r="I10" s="26"/>
       <c r="J10" s="26"/>
-      <c r="K10" s="66" t="s">
+      <c r="K10" s="69" t="s">
         <v>48</v>
       </c>
     </row>
@@ -3247,7 +3271,7 @@
       </c>
       <c r="I11" s="26"/>
       <c r="J11" s="26"/>
-      <c r="K11" s="66" t="s">
+      <c r="K11" s="69" t="s">
         <v>52</v>
       </c>
     </row>
@@ -3274,7 +3298,7 @@
       </c>
       <c r="I12" s="26"/>
       <c r="J12" s="26"/>
-      <c r="K12" s="66" t="s">
+      <c r="K12" s="69" t="s">
         <v>56</v>
       </c>
     </row>
@@ -3301,7 +3325,7 @@
       </c>
       <c r="I13" s="26"/>
       <c r="J13" s="26"/>
-      <c r="K13" s="66" t="s">
+      <c r="K13" s="69" t="s">
         <v>60</v>
       </c>
     </row>
@@ -3328,7 +3352,7 @@
       </c>
       <c r="I14" s="26"/>
       <c r="J14" s="26"/>
-      <c r="K14" s="66" t="s">
+      <c r="K14" s="69" t="s">
         <v>64</v>
       </c>
     </row>
@@ -3355,7 +3379,7 @@
       </c>
       <c r="I15" s="26"/>
       <c r="J15" s="26"/>
-      <c r="K15" s="66" t="s">
+      <c r="K15" s="69" t="s">
         <v>68</v>
       </c>
     </row>
@@ -3382,7 +3406,7 @@
       </c>
       <c r="I16" s="26"/>
       <c r="J16" s="26"/>
-      <c r="K16" s="66" t="s">
+      <c r="K16" s="69" t="s">
         <v>72</v>
       </c>
     </row>
@@ -3409,7 +3433,7 @@
       </c>
       <c r="I17" s="32"/>
       <c r="J17" s="32"/>
-      <c r="K17" s="67" t="s">
+      <c r="K17" s="70" t="s">
         <v>77</v>
       </c>
     </row>
@@ -3436,7 +3460,7 @@
       </c>
       <c r="I18" s="32"/>
       <c r="J18" s="32"/>
-      <c r="K18" s="67" t="s">
+      <c r="K18" s="70" t="s">
         <v>81</v>
       </c>
     </row>
@@ -3463,7 +3487,7 @@
       </c>
       <c r="I19" s="26"/>
       <c r="J19" s="26"/>
-      <c r="K19" s="68" t="s">
+      <c r="K19" s="71" t="s">
         <v>87</v>
       </c>
     </row>
@@ -3484,7 +3508,7 @@
       </c>
       <c r="I20" s="26"/>
       <c r="J20" s="26"/>
-      <c r="K20" s="69" t="s">
+      <c r="K20" s="72" t="s">
         <v>89</v>
       </c>
     </row>
@@ -3505,7 +3529,7 @@
       </c>
       <c r="I21" s="26"/>
       <c r="J21" s="26"/>
-      <c r="K21" s="69" t="s">
+      <c r="K21" s="72" t="s">
         <v>91</v>
       </c>
     </row>
@@ -3526,7 +3550,7 @@
       </c>
       <c r="I22" s="26"/>
       <c r="J22" s="26"/>
-      <c r="K22" s="69" t="s">
+      <c r="K22" s="72" t="s">
         <v>93</v>
       </c>
     </row>
@@ -3543,13 +3567,13 @@
       <c r="D23" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="E23" s="75" t="s">
+      <c r="E23" s="79" t="s">
         <v>98</v>
       </c>
-      <c r="F23" s="75" t="s">
+      <c r="F23" s="79" t="s">
         <v>99</v>
       </c>
-      <c r="G23" s="75" t="s">
+      <c r="G23" s="79" t="s">
         <v>100</v>
       </c>
       <c r="H23" s="23" t="s">
@@ -3557,7 +3581,7 @@
       </c>
       <c r="I23" s="26"/>
       <c r="J23" s="26"/>
-      <c r="K23" s="79" t="s">
+      <c r="K23" s="83" t="s">
         <v>102</v>
       </c>
     </row>
@@ -3573,7 +3597,7 @@
       </c>
       <c r="F24" s="26"/>
       <c r="G24" s="26"/>
-      <c r="H24" s="75" t="s">
+      <c r="H24" s="79" t="s">
         <v>104</v>
       </c>
       <c r="I24" s="22" t="s">
@@ -3582,7 +3606,7 @@
       <c r="J24" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="K24" s="64" t="s">
+      <c r="K24" s="67" t="s">
         <v>107</v>
       </c>
     </row>
@@ -3604,16 +3628,16 @@
       </c>
       <c r="F25" s="26"/>
       <c r="G25" s="26"/>
-      <c r="H25" s="75" t="s">
+      <c r="H25" s="79" t="s">
         <v>112</v>
       </c>
       <c r="I25" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="J25" s="80" t="s">
+      <c r="J25" s="84" t="s">
         <v>114</v>
       </c>
-      <c r="K25" s="64" t="s">
+      <c r="K25" s="67" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3629,16 +3653,16 @@
       </c>
       <c r="F26" s="26"/>
       <c r="G26" s="26"/>
-      <c r="H26" s="75" t="s">
+      <c r="H26" s="79" t="s">
         <v>117</v>
       </c>
       <c r="I26" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="J26" s="80" t="s">
+      <c r="J26" s="84" t="s">
         <v>119</v>
       </c>
-      <c r="K26" s="64" t="s">
+      <c r="K26" s="67" t="s">
         <v>120</v>
       </c>
     </row>
@@ -3655,13 +3679,13 @@
       <c r="D27" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="81" t="s">
+      <c r="E27" s="85" t="s">
         <v>124</v>
       </c>
       <c r="F27" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="G27" s="80" t="s">
+      <c r="G27" s="84" t="s">
         <v>125</v>
       </c>
       <c r="H27" s="23" t="s">
@@ -3669,7 +3693,7 @@
       </c>
       <c r="I27" s="26"/>
       <c r="J27" s="26"/>
-      <c r="K27" s="70" t="s">
+      <c r="K27" s="73" t="s">
         <v>126</v>
       </c>
     </row>
@@ -3696,7 +3720,7 @@
       </c>
       <c r="I28" s="41"/>
       <c r="J28" s="41"/>
-      <c r="K28" s="63"/>
+      <c r="K28" s="66"/>
     </row>
     <row r="29" ht="96" customHeight="1" spans="1:11">
       <c r="A29" s="42" t="s">
@@ -3711,7 +3735,7 @@
       <c r="D29" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="82" t="s">
+      <c r="E29" s="86" t="s">
         <v>134</v>
       </c>
       <c r="F29" s="44" t="s">
@@ -3725,7 +3749,7 @@
       </c>
       <c r="I29" s="26"/>
       <c r="J29" s="26"/>
-      <c r="K29" s="64" t="s">
+      <c r="K29" s="67" t="s">
         <v>136</v>
       </c>
     </row>
@@ -3741,16 +3765,16 @@
       </c>
       <c r="F30" s="26"/>
       <c r="G30" s="26"/>
-      <c r="H30" s="75" t="s">
+      <c r="H30" s="79" t="s">
         <v>138</v>
       </c>
       <c r="I30" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="J30" s="75" t="s">
+      <c r="J30" s="79" t="s">
         <v>140</v>
       </c>
-      <c r="K30" s="64" t="s">
+      <c r="K30" s="67" t="s">
         <v>141</v>
       </c>
     </row>
@@ -3764,7 +3788,7 @@
       <c r="E31" s="23"/>
       <c r="F31" s="26"/>
       <c r="G31" s="26"/>
-      <c r="H31" s="75" t="s">
+      <c r="H31" s="79" t="s">
         <v>143</v>
       </c>
       <c r="I31" s="22" t="s">
@@ -3773,7 +3797,7 @@
       <c r="J31" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="K31" s="64" t="s">
+      <c r="K31" s="67" t="s">
         <v>145</v>
       </c>
     </row>
@@ -3800,7 +3824,7 @@
       </c>
       <c r="I32" s="26"/>
       <c r="J32" s="26"/>
-      <c r="K32" s="63" t="s">
+      <c r="K32" s="66" t="s">
         <v>150</v>
       </c>
     </row>
@@ -3831,7 +3855,7 @@
       </c>
       <c r="I33" s="26"/>
       <c r="J33" s="26"/>
-      <c r="K33" s="63" t="s">
+      <c r="K33" s="66" t="s">
         <v>158</v>
       </c>
     </row>
@@ -3856,30 +3880,30 @@
       <c r="H34" s="48"/>
       <c r="I34" s="48"/>
       <c r="J34" s="48"/>
-      <c r="K34" s="71"/>
+      <c r="K34" s="74"/>
     </row>
     <row r="35" ht="31.2" spans="1:11">
       <c r="A35" s="50" t="s">
         <v>164</v>
       </c>
-      <c r="B35" s="48" t="s">
+      <c r="B35" s="51" t="s">
         <v>165</v>
       </c>
-      <c r="C35" s="48" t="s">
+      <c r="C35" s="51" t="s">
         <v>166</v>
       </c>
-      <c r="D35" s="49" t="s">
+      <c r="D35" s="52" t="s">
         <v>162</v>
       </c>
-      <c r="E35" s="48" t="s">
+      <c r="E35" s="51" t="s">
         <v>163</v>
       </c>
-      <c r="F35" s="48"/>
-      <c r="G35" s="48"/>
-      <c r="H35" s="48"/>
-      <c r="I35" s="48"/>
-      <c r="J35" s="48"/>
-      <c r="K35" s="71"/>
+      <c r="F35" s="51"/>
+      <c r="G35" s="51"/>
+      <c r="H35" s="51"/>
+      <c r="I35" s="51"/>
+      <c r="J35" s="51"/>
+      <c r="K35" s="75"/>
     </row>
     <row r="36" ht="31.2" spans="1:11">
       <c r="A36" s="35" t="s">
@@ -3891,13 +3915,13 @@
       <c r="C36" s="36" t="s">
         <v>169</v>
       </c>
-      <c r="D36" s="51" t="s">
+      <c r="D36" s="53" t="s">
         <v>170</v>
       </c>
-      <c r="E36" s="52" t="s">
+      <c r="E36" s="54" t="s">
         <v>171</v>
       </c>
-      <c r="F36" s="83" t="s">
+      <c r="F36" s="87" t="s">
         <v>172</v>
       </c>
       <c r="G36" s="36" t="s">
@@ -3908,7 +3932,7 @@
       </c>
       <c r="I36" s="26"/>
       <c r="J36" s="26"/>
-      <c r="K36" s="72" t="s">
+      <c r="K36" s="76" t="s">
         <v>174</v>
       </c>
     </row>
@@ -3916,7 +3940,7 @@
       <c r="A37" s="35"/>
       <c r="B37" s="36"/>
       <c r="C37" s="36"/>
-      <c r="D37" s="53" t="s">
+      <c r="D37" s="55" t="s">
         <v>175</v>
       </c>
       <c r="E37" s="23" t="s">
@@ -3933,7 +3957,7 @@
       <c r="J37" s="36" t="s">
         <v>178</v>
       </c>
-      <c r="K37" s="65" t="s">
+      <c r="K37" s="68" t="s">
         <v>179</v>
       </c>
     </row>
@@ -3941,7 +3965,7 @@
       <c r="A38" s="35"/>
       <c r="B38" s="36"/>
       <c r="C38" s="36"/>
-      <c r="D38" s="51" t="s">
+      <c r="D38" s="53" t="s">
         <v>180</v>
       </c>
       <c r="E38" s="23" t="s">
@@ -3949,16 +3973,16 @@
       </c>
       <c r="F38" s="26"/>
       <c r="G38" s="26"/>
-      <c r="H38" s="52" t="s">
+      <c r="H38" s="54" t="s">
         <v>181</v>
       </c>
-      <c r="I38" s="83" t="s">
+      <c r="I38" s="87" t="s">
         <v>172</v>
       </c>
       <c r="J38" s="36" t="s">
         <v>173</v>
       </c>
-      <c r="K38" s="65" t="s">
+      <c r="K38" s="68" t="s">
         <v>182</v>
       </c>
     </row>
@@ -3972,7 +3996,7 @@
       <c r="C39" s="36" t="s">
         <v>185</v>
       </c>
-      <c r="D39" s="51" t="s">
+      <c r="D39" s="53" t="s">
         <v>186</v>
       </c>
       <c r="E39" s="23" t="s">
@@ -3980,16 +4004,16 @@
       </c>
       <c r="F39" s="26"/>
       <c r="G39" s="26"/>
-      <c r="H39" s="52" t="s">
+      <c r="H39" s="54" t="s">
         <v>187</v>
       </c>
       <c r="I39" s="22" t="s">
         <v>188</v>
       </c>
-      <c r="J39" s="52" t="s">
+      <c r="J39" s="54" t="s">
         <v>189</v>
       </c>
-      <c r="K39" s="65" t="s">
+      <c r="K39" s="68" t="s">
         <v>190</v>
       </c>
     </row>
@@ -3997,16 +4021,16 @@
       <c r="A40" s="35"/>
       <c r="B40" s="36"/>
       <c r="C40" s="36"/>
-      <c r="D40" s="51" t="s">
+      <c r="D40" s="53" t="s">
         <v>191</v>
       </c>
       <c r="E40" s="36" t="s">
         <v>192</v>
       </c>
-      <c r="F40" s="52" t="s">
+      <c r="F40" s="54" t="s">
         <v>193</v>
       </c>
-      <c r="G40" s="54" t="s">
+      <c r="G40" s="56" t="s">
         <v>194</v>
       </c>
       <c r="H40" s="23" t="s">
@@ -4014,7 +4038,7 @@
       </c>
       <c r="I40" s="26"/>
       <c r="J40" s="26"/>
-      <c r="K40" s="73" t="s">
+      <c r="K40" s="77" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4022,16 +4046,16 @@
       <c r="A41" s="35"/>
       <c r="B41" s="36"/>
       <c r="C41" s="36"/>
-      <c r="D41" s="51" t="s">
+      <c r="D41" s="53" t="s">
         <v>196</v>
       </c>
-      <c r="E41" s="52" t="s">
+      <c r="E41" s="54" t="s">
         <v>197</v>
       </c>
-      <c r="F41" s="52" t="s">
+      <c r="F41" s="54" t="s">
         <v>193</v>
       </c>
-      <c r="G41" s="54" t="s">
+      <c r="G41" s="56" t="s">
         <v>198</v>
       </c>
       <c r="H41" s="23" t="s">
@@ -4039,7 +4063,7 @@
       </c>
       <c r="I41" s="26"/>
       <c r="J41" s="26"/>
-      <c r="K41" s="73" t="s">
+      <c r="K41" s="77" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4047,7 +4071,7 @@
       <c r="A42" s="35"/>
       <c r="B42" s="36"/>
       <c r="C42" s="36"/>
-      <c r="D42" s="51" t="s">
+      <c r="D42" s="53" t="s">
         <v>199</v>
       </c>
       <c r="E42" s="23" t="s">
@@ -4055,16 +4079,16 @@
       </c>
       <c r="F42" s="26"/>
       <c r="G42" s="26"/>
-      <c r="H42" s="52" t="s">
+      <c r="H42" s="54" t="s">
         <v>200</v>
       </c>
       <c r="I42" s="36" t="s">
         <v>201</v>
       </c>
-      <c r="J42" s="52" t="s">
+      <c r="J42" s="54" t="s">
         <v>202</v>
       </c>
-      <c r="K42" s="65" t="s">
+      <c r="K42" s="68" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4078,16 +4102,16 @@
       <c r="C43" s="36" t="s">
         <v>206</v>
       </c>
-      <c r="D43" s="51" t="s">
+      <c r="D43" s="53" t="s">
         <v>207</v>
       </c>
       <c r="E43" s="36" t="s">
         <v>208</v>
       </c>
-      <c r="F43" s="55" t="s">
+      <c r="F43" s="57" t="s">
         <v>165</v>
       </c>
-      <c r="G43" s="52" t="s">
+      <c r="G43" s="54" t="s">
         <v>209</v>
       </c>
       <c r="H43" s="23" t="s">
@@ -4095,7 +4119,7 @@
       </c>
       <c r="I43" s="26"/>
       <c r="J43" s="26"/>
-      <c r="K43" s="65" t="s">
+      <c r="K43" s="68" t="s">
         <v>210</v>
       </c>
     </row>
@@ -4103,28 +4127,28 @@
       <c r="A44" s="35"/>
       <c r="B44" s="36"/>
       <c r="C44" s="36"/>
-      <c r="D44" s="51" t="s">
+      <c r="D44" s="53" t="s">
         <v>211</v>
       </c>
       <c r="E44" s="36" t="s">
         <v>212</v>
       </c>
-      <c r="F44" s="55" t="s">
+      <c r="F44" s="57" t="s">
         <v>165</v>
       </c>
-      <c r="G44" s="52" t="s">
+      <c r="G44" s="54" t="s">
         <v>213</v>
       </c>
       <c r="H44" s="36" t="s">
         <v>214</v>
       </c>
-      <c r="I44" s="52" t="s">
+      <c r="I44" s="54" t="s">
         <v>215</v>
       </c>
       <c r="J44" s="36" t="s">
         <v>216</v>
       </c>
-      <c r="K44" s="65" t="s">
+      <c r="K44" s="68" t="s">
         <v>217</v>
       </c>
     </row>
@@ -4132,16 +4156,16 @@
       <c r="A45" s="35"/>
       <c r="B45" s="36"/>
       <c r="C45" s="36"/>
-      <c r="D45" s="51" t="s">
+      <c r="D45" s="53" t="s">
         <v>218</v>
       </c>
       <c r="E45" s="36" t="s">
         <v>219</v>
       </c>
-      <c r="F45" s="55" t="s">
+      <c r="F45" s="57" t="s">
         <v>165</v>
       </c>
-      <c r="G45" s="52" t="s">
+      <c r="G45" s="54" t="s">
         <v>220</v>
       </c>
       <c r="H45" s="23" t="s">
@@ -4149,7 +4173,7 @@
       </c>
       <c r="I45" s="26"/>
       <c r="J45" s="26"/>
-      <c r="K45" s="65" t="s">
+      <c r="K45" s="68" t="s">
         <v>221</v>
       </c>
     </row>
@@ -4157,16 +4181,16 @@
       <c r="A46" s="35"/>
       <c r="B46" s="36"/>
       <c r="C46" s="36"/>
-      <c r="D46" s="51" t="s">
+      <c r="D46" s="53" t="s">
         <v>222</v>
       </c>
       <c r="E46" s="36" t="s">
         <v>223</v>
       </c>
-      <c r="F46" s="55" t="s">
+      <c r="F46" s="57" t="s">
         <v>165</v>
       </c>
-      <c r="G46" s="52" t="s">
+      <c r="G46" s="54" t="s">
         <v>224</v>
       </c>
       <c r="H46" s="23" t="s">
@@ -4174,41 +4198,64 @@
       </c>
       <c r="I46" s="26"/>
       <c r="J46" s="26"/>
-      <c r="K46" s="65" t="s">
+      <c r="K46" s="68" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="47" ht="328.35" spans="1:11">
-      <c r="A47" s="56"/>
-      <c r="B47" s="57"/>
-      <c r="C47" s="57"/>
-      <c r="D47" s="58" t="s">
+      <c r="A47" s="58"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="60" t="s">
         <v>226</v>
       </c>
-      <c r="E47" s="57" t="s">
+      <c r="E47" s="59" t="s">
         <v>227</v>
       </c>
-      <c r="F47" s="59" t="s">
+      <c r="F47" s="61" t="s">
         <v>165</v>
       </c>
-      <c r="G47" s="60" t="s">
+      <c r="G47" s="62" t="s">
         <v>228</v>
       </c>
-      <c r="H47" s="57" t="s">
+      <c r="H47" s="59" t="s">
         <v>229</v>
       </c>
-      <c r="I47" s="60" t="s">
+      <c r="I47" s="62" t="s">
         <v>230</v>
       </c>
-      <c r="J47" s="57" t="s">
+      <c r="J47" s="59" t="s">
         <v>231</v>
       </c>
-      <c r="K47" s="74" t="s">
+      <c r="K47" s="78" t="s">
         <v>232</v>
       </c>
     </row>
+    <row r="48" ht="31.2" spans="1:11">
+      <c r="A48" s="63" t="s">
+        <v>233</v>
+      </c>
+      <c r="B48" s="48" t="s">
+        <v>165</v>
+      </c>
+      <c r="C48" s="48" t="s">
+        <v>234</v>
+      </c>
+      <c r="D48" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E48" s="48" t="s">
+        <v>163</v>
+      </c>
+      <c r="F48" s="48"/>
+      <c r="G48" s="48"/>
+      <c r="H48" s="48"/>
+      <c r="I48" s="48"/>
+      <c r="J48" s="48"/>
+      <c r="K48" s="74"/>
+    </row>
   </sheetData>
-  <mergeCells count="84">
+  <mergeCells count="85">
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="H4:J4"/>
@@ -4264,6 +4311,7 @@
     <mergeCell ref="H43:J43"/>
     <mergeCell ref="H45:J45"/>
     <mergeCell ref="H46:J46"/>
+    <mergeCell ref="E48:K48"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="A5:A9"/>
     <mergeCell ref="A19:A22"/>

</xml_diff>

<commit_message>
version 48 - Integrate RAG AI Chatbot for conversation
</commit_message>
<xml_diff>
--- a/Documentation/API_Design/RESTFul_API.xlsx
+++ b/Documentation/API_Design/RESTFul_API.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="8280"/>
   </bookViews>
   <sheets>
     <sheet name="Server APIs" sheetId="3" r:id="rId1"/>
@@ -176,7 +176,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="240">
   <si>
     <t>RESTfull API</t>
   </si>
@@ -1499,6 +1499,21 @@
   </si>
   <si>
     <t>/api/admin/update_products_mysql</t>
+  </si>
+  <si>
+    <t>API 26:  AI Chat bot service</t>
+  </si>
+  <si>
+    <t>RAG_Chatbot</t>
+  </si>
+  <si>
+    <t>/api/rag_chatbot</t>
+  </si>
+  <si>
+    <t>Transmit user question to RAG Chatbot service and get feedback from LLM</t>
+  </si>
+  <si>
+    <t>AI_RAG_CHATBOT_URL</t>
   </si>
 </sst>
 </file>
@@ -1721,16 +1736,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
       <i/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
       <charset val="134"/>
     </font>
     <font>
@@ -2991,7 +3006,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.4"/>
   <cols>
     <col min="1" max="1" width="38.5833333333333" style="2" customWidth="1"/>
@@ -4254,8 +4269,37 @@
       <c r="J48" s="48"/>
       <c r="K48" s="74"/>
     </row>
+    <row r="49" ht="78.75" spans="1:11">
+      <c r="A49" s="35" t="s">
+        <v>235</v>
+      </c>
+      <c r="B49" s="19" t="s">
+        <v>236</v>
+      </c>
+      <c r="C49" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="D49" s="21"/>
+      <c r="E49" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="F49" s="26"/>
+      <c r="G49" s="26"/>
+      <c r="H49" s="59" t="s">
+        <v>238</v>
+      </c>
+      <c r="I49" s="62" t="s">
+        <v>230</v>
+      </c>
+      <c r="J49" s="59" t="s">
+        <v>231</v>
+      </c>
+      <c r="K49" s="67" t="s">
+        <v>239</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="85">
+  <mergeCells count="86">
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="H4:J4"/>
@@ -4312,6 +4356,7 @@
     <mergeCell ref="H45:J45"/>
     <mergeCell ref="H46:J46"/>
     <mergeCell ref="E48:K48"/>
+    <mergeCell ref="E49:G49"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="A5:A9"/>
     <mergeCell ref="A19:A22"/>

</xml_diff>